<commit_message>
docs(QA, escenario de calidad y tácticas de arq)
</commit_message>
<xml_diff>
--- a/docs/Análisis de Requerimientos/Matriz Requerimientos.xlsx
+++ b/docs/Análisis de Requerimientos/Matriz Requerimientos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luxua\Documents\Proyects\Acciones-ElBosque\docs\Análisis de Requerimientos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D76B4B61-4F35-4B93-8E7E-75ACD41F8441}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D1F700D-B384-4369-B47A-7F8565557198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requerimientos Funcionales" sheetId="1" r:id="rId1"/>
@@ -735,19 +735,6 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -779,6 +766,19 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1098,32 +1098,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
     </row>
     <row r="2" spans="1:10" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="19"/>
     </row>
     <row r="3" spans="1:10" ht="63.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -1161,7 +1161,7 @@
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="B4" s="16" t="s">
         <v>65</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -1533,13 +1533,13 @@
       <c r="A16" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="21" t="s">
+      <c r="B16" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="C16" s="21" t="s">
+      <c r="C16" s="16" t="s">
         <v>124</v>
       </c>
-      <c r="D16" s="21" t="s">
+      <c r="D16" s="16" t="s">
         <v>83</v>
       </c>
       <c r="E16" s="2" t="s">
@@ -1551,7 +1551,7 @@
       <c r="G16" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="H16" s="21" t="s">
+      <c r="H16" s="16" t="s">
         <v>127</v>
       </c>
       <c r="I16" s="2" t="s">
@@ -1563,121 +1563,121 @@
       <c r="A17" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="15" t="s">
+      <c r="B17" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="C17" s="15" t="s">
+      <c r="C17" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="D17" s="15" t="s">
+      <c r="D17" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="E17" s="15" t="s">
+      <c r="E17" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="F17" s="15" t="s">
+      <c r="F17" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="G17" s="15" t="s">
+      <c r="G17" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="H17" s="15" t="s">
+      <c r="H17" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="I17" s="15" t="s">
+      <c r="I17" s="10" t="s">
         <v>85</v>
       </c>
       <c r="J17" s="4"/>
     </row>
     <row r="18" spans="1:10" ht="93.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="12" t="s">
         <v>129</v>
       </c>
-      <c r="C18" s="17" t="s">
+      <c r="C18" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="D18" s="17" t="s">
+      <c r="D18" s="12" t="s">
         <v>132</v>
       </c>
-      <c r="E18" s="17" t="s">
+      <c r="E18" s="12" t="s">
         <v>136</v>
       </c>
-      <c r="F18" s="17" t="s">
+      <c r="F18" s="12" t="s">
         <v>118</v>
       </c>
-      <c r="G18" s="17" t="s">
+      <c r="G18" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="H18" s="17" t="s">
+      <c r="H18" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="I18" s="17" t="s">
+      <c r="I18" s="12" t="s">
         <v>131</v>
       </c>
-      <c r="J18" s="12"/>
+      <c r="J18" s="7"/>
     </row>
     <row r="19" spans="1:10" ht="89.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="18" t="s">
+      <c r="A19" s="13" t="s">
         <v>122</v>
       </c>
-      <c r="B19" s="19" t="s">
+      <c r="B19" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="C19" s="19" t="s">
+      <c r="C19" s="14" t="s">
         <v>134</v>
       </c>
-      <c r="D19" s="19" t="s">
+      <c r="D19" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="E19" s="19" t="s">
+      <c r="E19" s="14" t="s">
         <v>137</v>
       </c>
-      <c r="F19" s="19" t="s">
+      <c r="F19" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="G19" s="18" t="s">
+      <c r="G19" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="H19" s="19" t="s">
+      <c r="H19" s="14" t="s">
         <v>139</v>
       </c>
-      <c r="I19" s="19" t="s">
+      <c r="I19" s="14" t="s">
         <v>131</v>
       </c>
-      <c r="J19" s="20"/>
+      <c r="J19" s="15"/>
     </row>
     <row r="20" spans="1:10" ht="85.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="16" t="s">
+      <c r="A20" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="B20" s="22" t="s">
+      <c r="B20" s="17" t="s">
         <v>140</v>
       </c>
-      <c r="C20" s="22" t="s">
+      <c r="C20" s="17" t="s">
         <v>141</v>
       </c>
-      <c r="D20" s="22" t="s">
+      <c r="D20" s="17" t="s">
         <v>142</v>
       </c>
-      <c r="E20" s="16" t="s">
+      <c r="E20" s="11" t="s">
         <v>143</v>
       </c>
-      <c r="F20" s="16" t="s">
+      <c r="F20" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="G20" s="16" t="s">
+      <c r="G20" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="H20" s="22" t="s">
+      <c r="H20" s="17" t="s">
         <v>138</v>
       </c>
-      <c r="I20" s="16" t="s">
+      <c r="I20" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="J20" s="16"/>
+      <c r="J20" s="11"/>
     </row>
     <row r="21" spans="1:10" ht="16.05" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="22" spans="1:10" ht="24.6" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -1685,98 +1685,98 @@
     <row r="24" spans="1:10" ht="16.05" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="25" spans="1:10" ht="16.05" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="37" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A37" s="10" t="s">
+      <c r="A37" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="B37" s="8"/>
-      <c r="C37" s="8"/>
-      <c r="D37" s="8"/>
-      <c r="E37" s="8"/>
-      <c r="F37" s="8"/>
-      <c r="G37" s="8"/>
-      <c r="H37" s="8"/>
-      <c r="I37" s="8"/>
-      <c r="J37" s="8"/>
+      <c r="B37" s="19"/>
+      <c r="C37" s="19"/>
+      <c r="D37" s="19"/>
+      <c r="E37" s="19"/>
+      <c r="F37" s="19"/>
+      <c r="G37" s="19"/>
+      <c r="H37" s="19"/>
+      <c r="I37" s="19"/>
+      <c r="J37" s="19"/>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B38" s="7" t="s">
+      <c r="B38" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="C38" s="8"/>
-      <c r="D38" s="8"/>
-      <c r="E38" s="8"/>
-      <c r="F38" s="8"/>
-      <c r="G38" s="8"/>
-      <c r="H38" s="8"/>
-      <c r="I38" s="8"/>
-      <c r="J38" s="8"/>
+      <c r="C38" s="19"/>
+      <c r="D38" s="19"/>
+      <c r="E38" s="19"/>
+      <c r="F38" s="19"/>
+      <c r="G38" s="19"/>
+      <c r="H38" s="19"/>
+      <c r="I38" s="19"/>
+      <c r="J38" s="19"/>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B39" s="7" t="s">
+      <c r="B39" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="C39" s="8"/>
-      <c r="D39" s="8"/>
-      <c r="E39" s="8"/>
-      <c r="F39" s="8"/>
-      <c r="G39" s="8"/>
-      <c r="H39" s="8"/>
-      <c r="I39" s="8"/>
-      <c r="J39" s="8"/>
+      <c r="C39" s="19"/>
+      <c r="D39" s="19"/>
+      <c r="E39" s="19"/>
+      <c r="F39" s="19"/>
+      <c r="G39" s="19"/>
+      <c r="H39" s="19"/>
+      <c r="I39" s="19"/>
+      <c r="J39" s="19"/>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B40" s="7" t="s">
+      <c r="B40" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="C40" s="8"/>
-      <c r="D40" s="8"/>
-      <c r="E40" s="8"/>
-      <c r="F40" s="8"/>
-      <c r="G40" s="8"/>
-      <c r="H40" s="8"/>
-      <c r="I40" s="8"/>
-      <c r="J40" s="8"/>
+      <c r="C40" s="19"/>
+      <c r="D40" s="19"/>
+      <c r="E40" s="19"/>
+      <c r="F40" s="19"/>
+      <c r="G40" s="19"/>
+      <c r="H40" s="19"/>
+      <c r="I40" s="19"/>
+      <c r="J40" s="19"/>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B41" s="7" t="s">
+      <c r="B41" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="C41" s="8"/>
-      <c r="D41" s="8"/>
-      <c r="E41" s="8"/>
-      <c r="F41" s="8"/>
-      <c r="G41" s="8"/>
-      <c r="H41" s="8"/>
-      <c r="I41" s="8"/>
-      <c r="J41" s="8"/>
+      <c r="C41" s="19"/>
+      <c r="D41" s="19"/>
+      <c r="E41" s="19"/>
+      <c r="F41" s="19"/>
+      <c r="G41" s="19"/>
+      <c r="H41" s="19"/>
+      <c r="I41" s="19"/>
+      <c r="J41" s="19"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B42" s="7" t="s">
+      <c r="B42" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="C42" s="8"/>
-      <c r="D42" s="8"/>
-      <c r="E42" s="8"/>
-      <c r="F42" s="8"/>
-      <c r="G42" s="8"/>
-      <c r="H42" s="8"/>
-      <c r="I42" s="8"/>
-      <c r="J42" s="8"/>
+      <c r="C42" s="19"/>
+      <c r="D42" s="19"/>
+      <c r="E42" s="19"/>
+      <c r="F42" s="19"/>
+      <c r="G42" s="19"/>
+      <c r="H42" s="19"/>
+      <c r="I42" s="19"/>
+      <c r="J42" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -1810,30 +1810,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
     </row>
     <row r="2" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="22" t="s">
         <v>166</v>
       </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
     </row>
     <row r="3" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -1868,7 +1868,7 @@
       <c r="A4" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="8" t="s">
         <v>145</v>
       </c>
       <c r="C4" s="3" t="s">
@@ -1897,7 +1897,7 @@
       <c r="A5" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="9" t="s">
         <v>144</v>
       </c>
       <c r="C5" s="5" t="s">
@@ -1924,7 +1924,7 @@
       <c r="A6" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="8" t="s">
         <v>144</v>
       </c>
       <c r="C6" s="3" t="s">
@@ -1949,7 +1949,7 @@
       <c r="A7" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="9" t="s">
         <v>146</v>
       </c>
       <c r="C7" s="5" t="s">
@@ -2142,92 +2142,92 @@
       <c r="I18" s="3"/>
     </row>
     <row r="20" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
+      <c r="B20" s="19"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="19"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="19"/>
     </row>
     <row r="21" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="C21" s="8"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8"/>
-      <c r="H21" s="8"/>
-      <c r="I21" s="8"/>
+      <c r="C21" s="19"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="19"/>
+      <c r="F21" s="19"/>
+      <c r="G21" s="19"/>
+      <c r="H21" s="19"/>
+      <c r="I21" s="19"/>
     </row>
     <row r="22" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
-      <c r="H22" s="8"/>
-      <c r="I22" s="8"/>
+      <c r="C22" s="19"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="19"/>
+      <c r="F22" s="19"/>
+      <c r="G22" s="19"/>
+      <c r="H22" s="19"/>
+      <c r="I22" s="19"/>
     </row>
     <row r="23" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="B23" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="C23" s="8"/>
-      <c r="D23" s="8"/>
-      <c r="E23" s="8"/>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
-      <c r="H23" s="8"/>
-      <c r="I23" s="8"/>
+      <c r="C23" s="19"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="19"/>
+      <c r="F23" s="19"/>
+      <c r="G23" s="19"/>
+      <c r="H23" s="19"/>
+      <c r="I23" s="19"/>
     </row>
     <row r="24" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="C24" s="8"/>
-      <c r="D24" s="8"/>
-      <c r="E24" s="8"/>
-      <c r="F24" s="8"/>
-      <c r="G24" s="8"/>
-      <c r="H24" s="8"/>
-      <c r="I24" s="8"/>
+      <c r="C24" s="19"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="19"/>
+      <c r="F24" s="19"/>
+      <c r="G24" s="19"/>
+      <c r="H24" s="19"/>
+      <c r="I24" s="19"/>
     </row>
     <row r="25" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="C25" s="8"/>
-      <c r="D25" s="8"/>
-      <c r="E25" s="8"/>
-      <c r="F25" s="8"/>
-      <c r="G25" s="8"/>
-      <c r="H25" s="8"/>
-      <c r="I25" s="8"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="19"/>
+      <c r="F25" s="19"/>
+      <c r="G25" s="19"/>
+      <c r="H25" s="19"/>
+      <c r="I25" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>